<commit_message>
Corrections suite aux revues+implémentation du mapping CDA/FHIR c6fb335d313740799b80ffbaa33bc0f0dc2947c6
</commit_message>
<xml_diff>
--- a/htr-FHIR/ig/StructureDefinition-DestinatairePrevu.xlsx
+++ b/htr-FHIR/ig/StructureDefinition-DestinatairePrevu.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-14T15:47:10+00:00</t>
+    <t>2025-03-25T13:52:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -249,7 +249,7 @@
     <t>Base</t>
   </si>
   <si>
-    <t>DestinatairePrevu.Destinataire</t>
+    <t>DestinatairePrevu.destinataire</t>
   </si>
   <si>
     <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/PersonneStructure
@@ -561,8 +561,8 @@
   <dimension ref="A1:AJ3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="29.34375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="29.34375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="29.09765625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="29.09765625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="12.66015625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="8.95703125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="6.77734375" customWidth="true" bestFit="true"/>
@@ -592,7 +592,7 @@
     <col min="29" max="29" width="20.59375" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="17.21484375" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="14.4140625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="29.34375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="29.09765625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="10.5546875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="11.0390625" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>

</xml_diff>